<commit_message>
GITBOOK-40: GITBOOK: trigger sync after projectDirectory update
</commit_message>
<xml_diff>
--- a/docs/0OMsoqOg9GiJ2xusVHMv/.gitbook/assets/IO - Template servizi - Canone unico patrimoniale (1).xlsx
+++ b/docs/0OMsoqOg9GiJ2xusVHMv/.gitbook/assets/IO - Template servizi - Canone unico patrimoniale (1).xlsx
@@ -559,7 +559,7 @@
         <rFont val="Titillium Web"/>
       </rPr>
       <t xml:space="preserve">
-Puoi pagare direttamente in app premendo “Paga”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
+Puoi pagare direttamente in app premendo “Vedi Avviso”, oppure tramite tutti i canali di pagamento della piattaforma pagoPA e le altre modalità di pagamento offerte dell'ente creditore.
 </t>
     </r>
     <r>
@@ -862,7 +862,7 @@
     <t>-</t>
   </si>
   <si>
-    <t>Paga (inserito automaticamente dall'app se il messaggio prevede un avviso di pagamento pagoPA)</t>
+    <t>Vedi Avviso</t>
   </si>
   <si>
     <t>Vedi ricevuta</t>

</xml_diff>